<commit_message>
Added the new sample file in master Data
</commit_message>
<xml_diff>
--- a/src/assets/Master_Data_Upload_template.xlsx
+++ b/src/assets/Master_Data_Upload_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sravanthi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC71E6B-89EE-458E-BB46-9CB71AE29F15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7796E5B7-C037-471D-A598-4E193584F331}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DropdownValues" sheetId="2" state="hidden" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="86">
   <si>
     <t>Type of Label</t>
   </si>
@@ -290,6 +290,12 @@
   </si>
   <si>
     <t>ethyl_code</t>
+  </si>
+  <si>
+    <t>Number of Color Settings</t>
+  </si>
+  <si>
+    <t>Number of Special Colors</t>
   </si>
 </sst>
 </file>
@@ -353,7 +359,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -376,12 +382,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -402,23 +419,14 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -725,164 +733,164 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A38"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>28</v>
       </c>
@@ -894,22 +902,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J100"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:L100"/>
+  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.54296875" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.81640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.26953125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="21.26953125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="6.90625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.21875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="21.21875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="6.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.77734375" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="4" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.1796875" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -940,8 +948,14 @@
       <c r="J1" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K1" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="L1" s="12" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
       <c r="B2" s="5"/>
       <c r="C2" s="2"/>
@@ -952,7 +966,7 @@
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -964,7 +978,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -976,7 +990,7 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -988,7 +1002,7 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -1000,7 +1014,7 @@
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -1012,7 +1026,7 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -1024,7 +1038,7 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -1036,7 +1050,7 @@
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1048,7 +1062,7 @@
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1060,7 +1074,7 @@
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -1072,7 +1086,7 @@
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -1084,7 +1098,7 @@
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -1096,7 +1110,7 @@
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1108,7 +1122,7 @@
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -1120,7 +1134,7 @@
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -1132,7 +1146,7 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -1144,7 +1158,7 @@
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1156,7 +1170,7 @@
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -1168,7 +1182,7 @@
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -1180,7 +1194,7 @@
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -1192,7 +1206,7 @@
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -1204,7 +1218,7 @@
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -1216,7 +1230,7 @@
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -1228,7 +1242,7 @@
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -1240,7 +1254,7 @@
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1252,7 +1266,7 @@
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1264,7 +1278,7 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1276,7 +1290,7 @@
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -1288,7 +1302,7 @@
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -1300,7 +1314,7 @@
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -1312,7 +1326,7 @@
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -1324,7 +1338,7 @@
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -1336,7 +1350,7 @@
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -1348,7 +1362,7 @@
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -1360,7 +1374,7 @@
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -1372,7 +1386,7 @@
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -1384,7 +1398,7 @@
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -1396,7 +1410,7 @@
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -1408,7 +1422,7 @@
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -1420,7 +1434,7 @@
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -1432,7 +1446,7 @@
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -1444,7 +1458,7 @@
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -1456,7 +1470,7 @@
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -1468,7 +1482,7 @@
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -1480,7 +1494,7 @@
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -1492,7 +1506,7 @@
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -1504,7 +1518,7 @@
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -1516,7 +1530,7 @@
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -1528,7 +1542,7 @@
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -1540,7 +1554,7 @@
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -1552,7 +1566,7 @@
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -1564,7 +1578,7 @@
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -1576,7 +1590,7 @@
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -1588,7 +1602,7 @@
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -1600,7 +1614,7 @@
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -1612,7 +1626,7 @@
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -1624,7 +1638,7 @@
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -1636,7 +1650,7 @@
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
@@ -1648,7 +1662,7 @@
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -1660,7 +1674,7 @@
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -1672,7 +1686,7 @@
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -1684,7 +1698,7 @@
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -1696,7 +1710,7 @@
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -1708,7 +1722,7 @@
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
@@ -1720,7 +1734,7 @@
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -1732,7 +1746,7 @@
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
@@ -1744,7 +1758,7 @@
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -1756,7 +1770,7 @@
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
@@ -1768,7 +1782,7 @@
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -1780,7 +1794,7 @@
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -1792,7 +1806,7 @@
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
@@ -1804,7 +1818,7 @@
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
@@ -1816,7 +1830,7 @@
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -1828,7 +1842,7 @@
       <c r="I75" s="2"/>
       <c r="J75" s="2"/>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
@@ -1840,7 +1854,7 @@
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -1852,7 +1866,7 @@
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -1864,7 +1878,7 @@
       <c r="I78" s="2"/>
       <c r="J78" s="2"/>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -1876,7 +1890,7 @@
       <c r="I79" s="2"/>
       <c r="J79" s="2"/>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -1888,7 +1902,7 @@
       <c r="I80" s="2"/>
       <c r="J80" s="2"/>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -1900,7 +1914,7 @@
       <c r="I81" s="2"/>
       <c r="J81" s="2"/>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
@@ -1912,7 +1926,7 @@
       <c r="I82" s="2"/>
       <c r="J82" s="2"/>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
@@ -1924,7 +1938,7 @@
       <c r="I83" s="2"/>
       <c r="J83" s="2"/>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -1936,7 +1950,7 @@
       <c r="I84" s="2"/>
       <c r="J84" s="2"/>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
@@ -1948,7 +1962,7 @@
       <c r="I85" s="2"/>
       <c r="J85" s="2"/>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -1960,7 +1974,7 @@
       <c r="I86" s="2"/>
       <c r="J86" s="2"/>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -1972,7 +1986,7 @@
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -1984,7 +1998,7 @@
       <c r="I88" s="2"/>
       <c r="J88" s="2"/>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -1996,7 +2010,7 @@
       <c r="I89" s="2"/>
       <c r="J89" s="2"/>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
@@ -2008,7 +2022,7 @@
       <c r="I90" s="2"/>
       <c r="J90" s="2"/>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -2020,7 +2034,7 @@
       <c r="I91" s="2"/>
       <c r="J91" s="2"/>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
@@ -2032,7 +2046,7 @@
       <c r="I92" s="2"/>
       <c r="J92" s="2"/>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -2044,7 +2058,7 @@
       <c r="I93" s="2"/>
       <c r="J93" s="2"/>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
@@ -2056,7 +2070,7 @@
       <c r="I94" s="2"/>
       <c r="J94" s="2"/>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -2068,7 +2082,7 @@
       <c r="I95" s="2"/>
       <c r="J95" s="2"/>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -2080,7 +2094,7 @@
       <c r="I96" s="2"/>
       <c r="J96" s="2"/>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -2092,7 +2106,7 @@
       <c r="I97" s="2"/>
       <c r="J97" s="2"/>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -2104,7 +2118,7 @@
       <c r="I98" s="2"/>
       <c r="J98" s="2"/>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -2116,7 +2130,7 @@
       <c r="I99" s="2"/>
       <c r="J99" s="2"/>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -2160,13 +2174,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:P100"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.1796875" style="2" customWidth="1"/>
-    <col min="2" max="16" width="20.81640625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="22.21875" style="2" customWidth="1"/>
+    <col min="2" max="16" width="20.77734375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -2216,7 +2230,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
       <c r="C2" s="2"/>
       <c r="D2" s="5"/>
@@ -2233,7 +2247,7 @@
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -2250,7 +2264,7 @@
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -2267,7 +2281,7 @@
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -2284,7 +2298,7 @@
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -2301,7 +2315,7 @@
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -2318,7 +2332,7 @@
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -2335,7 +2349,7 @@
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -2352,7 +2366,7 @@
       <c r="O9" s="2"/>
       <c r="P9" s="2"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -2369,7 +2383,7 @@
       <c r="O10" s="2"/>
       <c r="P10" s="2"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -2386,7 +2400,7 @@
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -2403,7 +2417,7 @@
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -2420,7 +2434,7 @@
       <c r="O13" s="2"/>
       <c r="P13" s="2"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -2437,7 +2451,7 @@
       <c r="O14" s="2"/>
       <c r="P14" s="2"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -2454,7 +2468,7 @@
       <c r="O15" s="2"/>
       <c r="P15" s="2"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -2471,7 +2485,7 @@
       <c r="O16" s="2"/>
       <c r="P16" s="2"/>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -2488,7 +2502,7 @@
       <c r="O17" s="2"/>
       <c r="P17" s="2"/>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -2505,7 +2519,7 @@
       <c r="O18" s="2"/>
       <c r="P18" s="2"/>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -2522,7 +2536,7 @@
       <c r="O19" s="2"/>
       <c r="P19" s="2"/>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -2539,7 +2553,7 @@
       <c r="O20" s="2"/>
       <c r="P20" s="2"/>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -2556,7 +2570,7 @@
       <c r="O21" s="2"/>
       <c r="P21" s="2"/>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -2573,7 +2587,7 @@
       <c r="O22" s="2"/>
       <c r="P22" s="2"/>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -2590,7 +2604,7 @@
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -2607,7 +2621,7 @@
       <c r="O24" s="2"/>
       <c r="P24" s="2"/>
     </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -2624,7 +2638,7 @@
       <c r="O25" s="2"/>
       <c r="P25" s="2"/>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -2641,7 +2655,7 @@
       <c r="O26" s="2"/>
       <c r="P26" s="2"/>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -2658,7 +2672,7 @@
       <c r="O27" s="2"/>
       <c r="P27" s="2"/>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -2675,7 +2689,7 @@
       <c r="O28" s="2"/>
       <c r="P28" s="2"/>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -2692,7 +2706,7 @@
       <c r="O29" s="2"/>
       <c r="P29" s="2"/>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -2709,7 +2723,7 @@
       <c r="O30" s="2"/>
       <c r="P30" s="2"/>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -2726,7 +2740,7 @@
       <c r="O31" s="2"/>
       <c r="P31" s="2"/>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -2743,7 +2757,7 @@
       <c r="O32" s="2"/>
       <c r="P32" s="2"/>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -2760,7 +2774,7 @@
       <c r="O33" s="2"/>
       <c r="P33" s="2"/>
     </row>
-    <row r="34" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -2777,7 +2791,7 @@
       <c r="O34" s="2"/>
       <c r="P34" s="2"/>
     </row>
-    <row r="35" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -2794,7 +2808,7 @@
       <c r="O35" s="2"/>
       <c r="P35" s="2"/>
     </row>
-    <row r="36" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -2811,7 +2825,7 @@
       <c r="O36" s="2"/>
       <c r="P36" s="2"/>
     </row>
-    <row r="37" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -2828,7 +2842,7 @@
       <c r="O37" s="2"/>
       <c r="P37" s="2"/>
     </row>
-    <row r="38" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
@@ -2845,7 +2859,7 @@
       <c r="O38" s="2"/>
       <c r="P38" s="2"/>
     </row>
-    <row r="39" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -2862,7 +2876,7 @@
       <c r="O39" s="2"/>
       <c r="P39" s="2"/>
     </row>
-    <row r="40" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -2879,7 +2893,7 @@
       <c r="O40" s="2"/>
       <c r="P40" s="2"/>
     </row>
-    <row r="41" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
@@ -2896,7 +2910,7 @@
       <c r="O41" s="2"/>
       <c r="P41" s="2"/>
     </row>
-    <row r="42" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
@@ -2913,7 +2927,7 @@
       <c r="O42" s="2"/>
       <c r="P42" s="2"/>
     </row>
-    <row r="43" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -2930,7 +2944,7 @@
       <c r="O43" s="2"/>
       <c r="P43" s="2"/>
     </row>
-    <row r="44" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
@@ -2947,7 +2961,7 @@
       <c r="O44" s="2"/>
       <c r="P44" s="2"/>
     </row>
-    <row r="45" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
@@ -2964,7 +2978,7 @@
       <c r="O45" s="2"/>
       <c r="P45" s="2"/>
     </row>
-    <row r="46" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
@@ -2981,7 +2995,7 @@
       <c r="O46" s="2"/>
       <c r="P46" s="2"/>
     </row>
-    <row r="47" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
@@ -2998,7 +3012,7 @@
       <c r="O47" s="2"/>
       <c r="P47" s="2"/>
     </row>
-    <row r="48" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -3015,7 +3029,7 @@
       <c r="O48" s="2"/>
       <c r="P48" s="2"/>
     </row>
-    <row r="49" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
@@ -3032,7 +3046,7 @@
       <c r="O49" s="2"/>
       <c r="P49" s="2"/>
     </row>
-    <row r="50" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
@@ -3049,7 +3063,7 @@
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
     </row>
-    <row r="51" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
@@ -3066,7 +3080,7 @@
       <c r="O51" s="2"/>
       <c r="P51" s="2"/>
     </row>
-    <row r="52" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
@@ -3083,7 +3097,7 @@
       <c r="O52" s="2"/>
       <c r="P52" s="2"/>
     </row>
-    <row r="53" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
@@ -3100,7 +3114,7 @@
       <c r="O53" s="2"/>
       <c r="P53" s="2"/>
     </row>
-    <row r="54" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
@@ -3117,7 +3131,7 @@
       <c r="O54" s="2"/>
       <c r="P54" s="2"/>
     </row>
-    <row r="55" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
@@ -3134,7 +3148,7 @@
       <c r="O55" s="2"/>
       <c r="P55" s="2"/>
     </row>
-    <row r="56" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
@@ -3151,7 +3165,7 @@
       <c r="O56" s="2"/>
       <c r="P56" s="2"/>
     </row>
-    <row r="57" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
@@ -3168,7 +3182,7 @@
       <c r="O57" s="2"/>
       <c r="P57" s="2"/>
     </row>
-    <row r="58" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
@@ -3185,7 +3199,7 @@
       <c r="O58" s="2"/>
       <c r="P58" s="2"/>
     </row>
-    <row r="59" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
@@ -3202,7 +3216,7 @@
       <c r="O59" s="2"/>
       <c r="P59" s="2"/>
     </row>
-    <row r="60" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
@@ -3219,7 +3233,7 @@
       <c r="O60" s="2"/>
       <c r="P60" s="2"/>
     </row>
-    <row r="61" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
@@ -3236,7 +3250,7 @@
       <c r="O61" s="2"/>
       <c r="P61" s="2"/>
     </row>
-    <row r="62" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
@@ -3253,7 +3267,7 @@
       <c r="O62" s="2"/>
       <c r="P62" s="2"/>
     </row>
-    <row r="63" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
@@ -3270,7 +3284,7 @@
       <c r="O63" s="2"/>
       <c r="P63" s="2"/>
     </row>
-    <row r="64" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
@@ -3287,7 +3301,7 @@
       <c r="O64" s="2"/>
       <c r="P64" s="2"/>
     </row>
-    <row r="65" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
@@ -3304,7 +3318,7 @@
       <c r="O65" s="2"/>
       <c r="P65" s="2"/>
     </row>
-    <row r="66" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
@@ -3321,7 +3335,7 @@
       <c r="O66" s="2"/>
       <c r="P66" s="2"/>
     </row>
-    <row r="67" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
@@ -3338,7 +3352,7 @@
       <c r="O67" s="2"/>
       <c r="P67" s="2"/>
     </row>
-    <row r="68" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
       <c r="D68" s="2"/>
@@ -3355,7 +3369,7 @@
       <c r="O68" s="2"/>
       <c r="P68" s="2"/>
     </row>
-    <row r="69" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
       <c r="D69" s="2"/>
@@ -3372,7 +3386,7 @@
       <c r="O69" s="2"/>
       <c r="P69" s="2"/>
     </row>
-    <row r="70" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
       <c r="D70" s="2"/>
@@ -3389,7 +3403,7 @@
       <c r="O70" s="2"/>
       <c r="P70" s="2"/>
     </row>
-    <row r="71" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
       <c r="D71" s="2"/>
@@ -3406,7 +3420,7 @@
       <c r="O71" s="2"/>
       <c r="P71" s="2"/>
     </row>
-    <row r="72" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
       <c r="D72" s="2"/>
@@ -3423,7 +3437,7 @@
       <c r="O72" s="2"/>
       <c r="P72" s="2"/>
     </row>
-    <row r="73" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
       <c r="D73" s="2"/>
@@ -3440,7 +3454,7 @@
       <c r="O73" s="2"/>
       <c r="P73" s="2"/>
     </row>
-    <row r="74" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
       <c r="D74" s="2"/>
@@ -3457,7 +3471,7 @@
       <c r="O74" s="2"/>
       <c r="P74" s="2"/>
     </row>
-    <row r="75" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
@@ -3474,7 +3488,7 @@
       <c r="O75" s="2"/>
       <c r="P75" s="2"/>
     </row>
-    <row r="76" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
@@ -3491,7 +3505,7 @@
       <c r="O76" s="2"/>
       <c r="P76" s="2"/>
     </row>
-    <row r="77" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
       <c r="D77" s="2"/>
@@ -3508,7 +3522,7 @@
       <c r="O77" s="2"/>
       <c r="P77" s="2"/>
     </row>
-    <row r="78" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
@@ -3525,7 +3539,7 @@
       <c r="O78" s="2"/>
       <c r="P78" s="2"/>
     </row>
-    <row r="79" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
@@ -3542,7 +3556,7 @@
       <c r="O79" s="2"/>
       <c r="P79" s="2"/>
     </row>
-    <row r="80" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
@@ -3559,7 +3573,7 @@
       <c r="O80" s="2"/>
       <c r="P80" s="2"/>
     </row>
-    <row r="81" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
       <c r="D81" s="2"/>
@@ -3576,7 +3590,7 @@
       <c r="O81" s="2"/>
       <c r="P81" s="2"/>
     </row>
-    <row r="82" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
       <c r="D82" s="2"/>
@@ -3593,7 +3607,7 @@
       <c r="O82" s="2"/>
       <c r="P82" s="2"/>
     </row>
-    <row r="83" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
       <c r="D83" s="2"/>
@@ -3610,7 +3624,7 @@
       <c r="O83" s="2"/>
       <c r="P83" s="2"/>
     </row>
-    <row r="84" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
       <c r="D84" s="2"/>
@@ -3627,7 +3641,7 @@
       <c r="O84" s="2"/>
       <c r="P84" s="2"/>
     </row>
-    <row r="85" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
       <c r="D85" s="2"/>
@@ -3644,7 +3658,7 @@
       <c r="O85" s="2"/>
       <c r="P85" s="2"/>
     </row>
-    <row r="86" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
@@ -3661,7 +3675,7 @@
       <c r="O86" s="2"/>
       <c r="P86" s="2"/>
     </row>
-    <row r="87" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
@@ -3678,7 +3692,7 @@
       <c r="O87" s="2"/>
       <c r="P87" s="2"/>
     </row>
-    <row r="88" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
@@ -3695,7 +3709,7 @@
       <c r="O88" s="2"/>
       <c r="P88" s="2"/>
     </row>
-    <row r="89" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
@@ -3712,7 +3726,7 @@
       <c r="O89" s="2"/>
       <c r="P89" s="2"/>
     </row>
-    <row r="90" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
@@ -3729,7 +3743,7 @@
       <c r="O90" s="2"/>
       <c r="P90" s="2"/>
     </row>
-    <row r="91" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
       <c r="D91" s="2"/>
@@ -3746,7 +3760,7 @@
       <c r="O91" s="2"/>
       <c r="P91" s="2"/>
     </row>
-    <row r="92" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2"/>
@@ -3763,7 +3777,7 @@
       <c r="O92" s="2"/>
       <c r="P92" s="2"/>
     </row>
-    <row r="93" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
       <c r="D93" s="2"/>
@@ -3780,7 +3794,7 @@
       <c r="O93" s="2"/>
       <c r="P93" s="2"/>
     </row>
-    <row r="94" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
       <c r="D94" s="2"/>
@@ -3797,7 +3811,7 @@
       <c r="O94" s="2"/>
       <c r="P94" s="2"/>
     </row>
-    <row r="95" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
       <c r="D95" s="2"/>
@@ -3814,7 +3828,7 @@
       <c r="O95" s="2"/>
       <c r="P95" s="2"/>
     </row>
-    <row r="96" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
       <c r="D96" s="2"/>
@@ -3831,7 +3845,7 @@
       <c r="O96" s="2"/>
       <c r="P96" s="2"/>
     </row>
-    <row r="97" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
       <c r="D97" s="2"/>
@@ -3848,7 +3862,7 @@
       <c r="O97" s="2"/>
       <c r="P97" s="2"/>
     </row>
-    <row r="98" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
       <c r="D98" s="2"/>
@@ -3865,7 +3879,7 @@
       <c r="O98" s="2"/>
       <c r="P98" s="2"/>
     </row>
-    <row r="99" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
       <c r="D99" s="2"/>
@@ -3882,7 +3896,7 @@
       <c r="O99" s="2"/>
       <c r="P99" s="2"/>
     </row>
-    <row r="100" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
       <c r="D100" s="2"/>
@@ -3908,23 +3922,23 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:L100"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.1796875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.54296875" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.54296875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="8.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.21875" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="8.44140625" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8" style="3" customWidth="1"/>
     <col min="9" max="9" width="12" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.54296875" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.1796875" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.81640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.77734375" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -3962,7 +3976,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3973,7 +3987,7 @@
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -3984,7 +3998,7 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -3995,7 +4009,7 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -4006,7 +4020,7 @@
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -4017,7 +4031,7 @@
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4028,7 +4042,7 @@
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -4039,7 +4053,7 @@
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -4050,7 +4064,7 @@
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -4061,7 +4075,7 @@
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -4072,7 +4086,7 @@
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="9"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -4083,7 +4097,7 @@
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="9"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -4094,7 +4108,7 @@
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="9"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -4105,7 +4119,7 @@
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="9"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -4116,7 +4130,7 @@
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="9"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -4127,7 +4141,7 @@
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="9"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -4138,7 +4152,7 @@
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="9"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -4149,7 +4163,7 @@
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="9"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -4160,7 +4174,7 @@
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="9"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -4171,7 +4185,7 @@
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="9"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -4182,7 +4196,7 @@
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -4193,7 +4207,7 @@
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -4204,7 +4218,7 @@
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -4215,7 +4229,7 @@
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -4226,7 +4240,7 @@
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -4237,7 +4251,7 @@
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -4248,7 +4262,7 @@
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -4259,7 +4273,7 @@
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -4270,7 +4284,7 @@
       <c r="H29" s="2"/>
       <c r="I29" s="2"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -4281,7 +4295,7 @@
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -4292,7 +4306,7 @@
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -4303,7 +4317,7 @@
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -4314,7 +4328,7 @@
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -4325,7 +4339,7 @@
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -4336,7 +4350,7 @@
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -4347,7 +4361,7 @@
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -4358,7 +4372,7 @@
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -4369,7 +4383,7 @@
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -4380,7 +4394,7 @@
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -4391,7 +4405,7 @@
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -4402,7 +4416,7 @@
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -4413,7 +4427,7 @@
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -4424,7 +4438,7 @@
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -4435,7 +4449,7 @@
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -4446,7 +4460,7 @@
       <c r="H45" s="2"/>
       <c r="I45" s="2"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -4457,7 +4471,7 @@
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -4468,7 +4482,7 @@
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -4479,7 +4493,7 @@
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -4490,7 +4504,7 @@
       <c r="H49" s="2"/>
       <c r="I49" s="2"/>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -4501,7 +4515,7 @@
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -4512,7 +4526,7 @@
       <c r="H51" s="2"/>
       <c r="I51" s="2"/>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -4523,7 +4537,7 @@
       <c r="H52" s="2"/>
       <c r="I52" s="2"/>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -4534,7 +4548,7 @@
       <c r="H53" s="2"/>
       <c r="I53" s="2"/>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -4545,7 +4559,7 @@
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -4556,7 +4570,7 @@
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -4567,7 +4581,7 @@
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -4578,7 +4592,7 @@
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -4589,7 +4603,7 @@
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -4600,7 +4614,7 @@
       <c r="H59" s="2"/>
       <c r="I59" s="2"/>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
@@ -4611,7 +4625,7 @@
       <c r="H60" s="2"/>
       <c r="I60" s="2"/>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -4622,7 +4636,7 @@
       <c r="H61" s="2"/>
       <c r="I61" s="2"/>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -4633,7 +4647,7 @@
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -4644,7 +4658,7 @@
       <c r="H63" s="2"/>
       <c r="I63" s="2"/>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -4655,7 +4669,7 @@
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -4666,7 +4680,7 @@
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
@@ -4677,7 +4691,7 @@
       <c r="H66" s="2"/>
       <c r="I66" s="2"/>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -4688,7 +4702,7 @@
       <c r="H67" s="2"/>
       <c r="I67" s="2"/>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
@@ -4699,7 +4713,7 @@
       <c r="H68" s="2"/>
       <c r="I68" s="2"/>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -4710,7 +4724,7 @@
       <c r="H69" s="2"/>
       <c r="I69" s="2"/>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
@@ -4721,7 +4735,7 @@
       <c r="H70" s="2"/>
       <c r="I70" s="2"/>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -4732,7 +4746,7 @@
       <c r="H71" s="2"/>
       <c r="I71" s="2"/>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -4743,7 +4757,7 @@
       <c r="H72" s="2"/>
       <c r="I72" s="2"/>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
@@ -4754,7 +4768,7 @@
       <c r="H73" s="2"/>
       <c r="I73" s="2"/>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
@@ -4765,7 +4779,7 @@
       <c r="H74" s="2"/>
       <c r="I74" s="2"/>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -4776,7 +4790,7 @@
       <c r="H75" s="2"/>
       <c r="I75" s="2"/>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
@@ -4787,7 +4801,7 @@
       <c r="H76" s="2"/>
       <c r="I76" s="2"/>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -4798,7 +4812,7 @@
       <c r="H77" s="2"/>
       <c r="I77" s="2"/>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -4809,7 +4823,7 @@
       <c r="H78" s="2"/>
       <c r="I78" s="2"/>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -4820,7 +4834,7 @@
       <c r="H79" s="2"/>
       <c r="I79" s="2"/>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -4831,7 +4845,7 @@
       <c r="H80" s="2"/>
       <c r="I80" s="2"/>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -4842,7 +4856,7 @@
       <c r="H81" s="2"/>
       <c r="I81" s="2"/>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
@@ -4853,7 +4867,7 @@
       <c r="H82" s="2"/>
       <c r="I82" s="2"/>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
@@ -4864,7 +4878,7 @@
       <c r="H83" s="2"/>
       <c r="I83" s="2"/>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -4875,7 +4889,7 @@
       <c r="H84" s="2"/>
       <c r="I84" s="2"/>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
@@ -4886,7 +4900,7 @@
       <c r="H85" s="2"/>
       <c r="I85" s="2"/>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -4897,7 +4911,7 @@
       <c r="H86" s="2"/>
       <c r="I86" s="2"/>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -4908,7 +4922,7 @@
       <c r="H87" s="2"/>
       <c r="I87" s="2"/>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -4919,7 +4933,7 @@
       <c r="H88" s="2"/>
       <c r="I88" s="2"/>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -4930,7 +4944,7 @@
       <c r="H89" s="2"/>
       <c r="I89" s="2"/>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
@@ -4941,7 +4955,7 @@
       <c r="H90" s="2"/>
       <c r="I90" s="2"/>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -4952,7 +4966,7 @@
       <c r="H91" s="2"/>
       <c r="I91" s="2"/>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
@@ -4963,7 +4977,7 @@
       <c r="H92" s="2"/>
       <c r="I92" s="2"/>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -4974,7 +4988,7 @@
       <c r="H93" s="2"/>
       <c r="I93" s="2"/>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
@@ -4985,7 +4999,7 @@
       <c r="H94" s="2"/>
       <c r="I94" s="2"/>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -4996,7 +5010,7 @@
       <c r="H95" s="2"/>
       <c r="I95" s="2"/>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -5007,7 +5021,7 @@
       <c r="H96" s="2"/>
       <c r="I96" s="2"/>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -5018,7 +5032,7 @@
       <c r="H97" s="2"/>
       <c r="I97" s="2"/>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -5029,7 +5043,7 @@
       <c r="H98" s="2"/>
       <c r="I98" s="2"/>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -5040,7 +5054,7 @@
       <c r="H99" s="2"/>
       <c r="I99" s="2"/>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -5059,29 +5073,29 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:Z100"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="9" width="20.81640625" style="3" customWidth="1"/>
-    <col min="10" max="10" width="13.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.1796875" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.1796875" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.81640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.54296875" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.36328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.08984375" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.90625" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.81640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.81640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="9" width="20.77734375" style="3" customWidth="1"/>
+    <col min="10" max="10" width="13.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.21875" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.21875" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.77734375" style="2" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="12" style="2" customWidth="1"/>
-    <col min="21" max="21" width="9.1796875" style="2"/>
-    <col min="22" max="22" width="10.90625" style="2" customWidth="1"/>
-    <col min="23" max="23" width="11.6328125" style="2" customWidth="1"/>
+    <col min="21" max="21" width="9.21875" style="2"/>
+    <col min="22" max="22" width="10.88671875" style="2" customWidth="1"/>
+    <col min="23" max="23" width="11.6640625" style="2" customWidth="1"/>
     <col min="24" max="24" width="10" style="2" customWidth="1"/>
-    <col min="25" max="25" width="14.36328125" style="2" customWidth="1"/>
-    <col min="26" max="26" width="13.90625" style="2" customWidth="1"/>
+    <col min="25" max="25" width="14.33203125" style="2" customWidth="1"/>
+    <col min="26" max="26" width="13.88671875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:26" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -5161,63 +5175,55 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:26" s="16" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="10"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
-      <c r="P2" s="14"/>
-      <c r="Q2" s="14"/>
-      <c r="R2" s="13"/>
-      <c r="S2" s="14"/>
-      <c r="T2" s="14"/>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="15"/>
-      <c r="Z2" s="15"/>
-    </row>
-    <row r="3" spans="1:26" s="16" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="17"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="13"/>
-      <c r="S3" s="14"/>
-      <c r="T3" s="14"/>
-      <c r="U3" s="13"/>
-      <c r="V3" s="13"/>
-      <c r="W3" s="13"/>
-      <c r="X3" s="13"/>
-      <c r="Y3" s="15"/>
-      <c r="Z3" s="15"/>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="4"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
+    </row>
+    <row r="3" spans="1:26" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="9"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="Y3" s="11"/>
+      <c r="Z3" s="11"/>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -5237,7 +5243,7 @@
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -5257,7 +5263,7 @@
       <c r="Q5" s="2"/>
       <c r="R5" s="2"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -5277,7 +5283,7 @@
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -5297,7 +5303,7 @@
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -5317,7 +5323,7 @@
       <c r="Q8" s="2"/>
       <c r="R8" s="2"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -5337,7 +5343,7 @@
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -5357,7 +5363,7 @@
       <c r="Q10" s="2"/>
       <c r="R10" s="2"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -5377,7 +5383,7 @@
       <c r="Q11" s="2"/>
       <c r="R11" s="2"/>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -5397,7 +5403,7 @@
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -5417,7 +5423,7 @@
       <c r="Q13" s="2"/>
       <c r="R13" s="2"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -5437,7 +5443,7 @@
       <c r="Q14" s="2"/>
       <c r="R14" s="2"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -5457,7 +5463,7 @@
       <c r="Q15" s="2"/>
       <c r="R15" s="2"/>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -5477,7 +5483,7 @@
       <c r="Q16" s="2"/>
       <c r="R16" s="2"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -5497,7 +5503,7 @@
       <c r="Q17" s="2"/>
       <c r="R17" s="2"/>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -5517,7 +5523,7 @@
       <c r="Q18" s="2"/>
       <c r="R18" s="2"/>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -5537,7 +5543,7 @@
       <c r="Q19" s="2"/>
       <c r="R19" s="2"/>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -5557,7 +5563,7 @@
       <c r="Q20" s="2"/>
       <c r="R20" s="2"/>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -5577,7 +5583,7 @@
       <c r="Q21" s="2"/>
       <c r="R21" s="2"/>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -5597,7 +5603,7 @@
       <c r="Q22" s="2"/>
       <c r="R22" s="2"/>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -5617,7 +5623,7 @@
       <c r="Q23" s="2"/>
       <c r="R23" s="2"/>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -5637,7 +5643,7 @@
       <c r="Q24" s="2"/>
       <c r="R24" s="2"/>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -5657,7 +5663,7 @@
       <c r="Q25" s="2"/>
       <c r="R25" s="2"/>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -5677,7 +5683,7 @@
       <c r="Q26" s="2"/>
       <c r="R26" s="2"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -5697,7 +5703,7 @@
       <c r="Q27" s="2"/>
       <c r="R27" s="2"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -5717,7 +5723,7 @@
       <c r="Q28" s="2"/>
       <c r="R28" s="2"/>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -5737,7 +5743,7 @@
       <c r="Q29" s="2"/>
       <c r="R29" s="2"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -5757,7 +5763,7 @@
       <c r="Q30" s="2"/>
       <c r="R30" s="2"/>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -5777,7 +5783,7 @@
       <c r="Q31" s="2"/>
       <c r="R31" s="2"/>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -5797,7 +5803,7 @@
       <c r="Q32" s="2"/>
       <c r="R32" s="2"/>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -5817,7 +5823,7 @@
       <c r="Q33" s="2"/>
       <c r="R33" s="2"/>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -5837,7 +5843,7 @@
       <c r="Q34" s="2"/>
       <c r="R34" s="2"/>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -5857,7 +5863,7 @@
       <c r="Q35" s="2"/>
       <c r="R35" s="2"/>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -5877,7 +5883,7 @@
       <c r="Q36" s="2"/>
       <c r="R36" s="2"/>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -5897,7 +5903,7 @@
       <c r="Q37" s="2"/>
       <c r="R37" s="2"/>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -5917,7 +5923,7 @@
       <c r="Q38" s="2"/>
       <c r="R38" s="2"/>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -5937,7 +5943,7 @@
       <c r="Q39" s="2"/>
       <c r="R39" s="2"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -5957,7 +5963,7 @@
       <c r="Q40" s="2"/>
       <c r="R40" s="2"/>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -5977,7 +5983,7 @@
       <c r="Q41" s="2"/>
       <c r="R41" s="2"/>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -5997,7 +6003,7 @@
       <c r="Q42" s="2"/>
       <c r="R42" s="2"/>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -6017,7 +6023,7 @@
       <c r="Q43" s="2"/>
       <c r="R43" s="2"/>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -6037,7 +6043,7 @@
       <c r="Q44" s="2"/>
       <c r="R44" s="2"/>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -6057,7 +6063,7 @@
       <c r="Q45" s="2"/>
       <c r="R45" s="2"/>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -6077,7 +6083,7 @@
       <c r="Q46" s="2"/>
       <c r="R46" s="2"/>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -6097,7 +6103,7 @@
       <c r="Q47" s="2"/>
       <c r="R47" s="2"/>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -6117,7 +6123,7 @@
       <c r="Q48" s="2"/>
       <c r="R48" s="2"/>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -6137,7 +6143,7 @@
       <c r="Q49" s="2"/>
       <c r="R49" s="2"/>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -6157,7 +6163,7 @@
       <c r="Q50" s="2"/>
       <c r="R50" s="2"/>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -6177,7 +6183,7 @@
       <c r="Q51" s="2"/>
       <c r="R51" s="2"/>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -6197,7 +6203,7 @@
       <c r="Q52" s="2"/>
       <c r="R52" s="2"/>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -6217,7 +6223,7 @@
       <c r="Q53" s="2"/>
       <c r="R53" s="2"/>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -6237,7 +6243,7 @@
       <c r="Q54" s="2"/>
       <c r="R54" s="2"/>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -6257,7 +6263,7 @@
       <c r="Q55" s="2"/>
       <c r="R55" s="2"/>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -6277,7 +6283,7 @@
       <c r="Q56" s="2"/>
       <c r="R56" s="2"/>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -6297,7 +6303,7 @@
       <c r="Q57" s="2"/>
       <c r="R57" s="2"/>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -6317,7 +6323,7 @@
       <c r="Q58" s="2"/>
       <c r="R58" s="2"/>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -6337,7 +6343,7 @@
       <c r="Q59" s="2"/>
       <c r="R59" s="2"/>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
@@ -6357,7 +6363,7 @@
       <c r="Q60" s="2"/>
       <c r="R60" s="2"/>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -6377,7 +6383,7 @@
       <c r="Q61" s="2"/>
       <c r="R61" s="2"/>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -6397,7 +6403,7 @@
       <c r="Q62" s="2"/>
       <c r="R62" s="2"/>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -6417,7 +6423,7 @@
       <c r="Q63" s="2"/>
       <c r="R63" s="2"/>
     </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -6437,7 +6443,7 @@
       <c r="Q64" s="2"/>
       <c r="R64" s="2"/>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -6457,7 +6463,7 @@
       <c r="Q65" s="2"/>
       <c r="R65" s="2"/>
     </row>
-    <row r="66" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
@@ -6477,7 +6483,7 @@
       <c r="Q66" s="2"/>
       <c r="R66" s="2"/>
     </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -6497,7 +6503,7 @@
       <c r="Q67" s="2"/>
       <c r="R67" s="2"/>
     </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
@@ -6517,7 +6523,7 @@
       <c r="Q68" s="2"/>
       <c r="R68" s="2"/>
     </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -6537,7 +6543,7 @@
       <c r="Q69" s="2"/>
       <c r="R69" s="2"/>
     </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
@@ -6557,7 +6563,7 @@
       <c r="Q70" s="2"/>
       <c r="R70" s="2"/>
     </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -6577,7 +6583,7 @@
       <c r="Q71" s="2"/>
       <c r="R71" s="2"/>
     </row>
-    <row r="72" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -6597,7 +6603,7 @@
       <c r="Q72" s="2"/>
       <c r="R72" s="2"/>
     </row>
-    <row r="73" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
@@ -6617,7 +6623,7 @@
       <c r="Q73" s="2"/>
       <c r="R73" s="2"/>
     </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
@@ -6637,7 +6643,7 @@
       <c r="Q74" s="2"/>
       <c r="R74" s="2"/>
     </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -6657,7 +6663,7 @@
       <c r="Q75" s="2"/>
       <c r="R75" s="2"/>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
@@ -6677,7 +6683,7 @@
       <c r="Q76" s="2"/>
       <c r="R76" s="2"/>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -6697,7 +6703,7 @@
       <c r="Q77" s="2"/>
       <c r="R77" s="2"/>
     </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -6717,7 +6723,7 @@
       <c r="Q78" s="2"/>
       <c r="R78" s="2"/>
     </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -6737,7 +6743,7 @@
       <c r="Q79" s="2"/>
       <c r="R79" s="2"/>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -6757,7 +6763,7 @@
       <c r="Q80" s="2"/>
       <c r="R80" s="2"/>
     </row>
-    <row r="81" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -6777,7 +6783,7 @@
       <c r="Q81" s="2"/>
       <c r="R81" s="2"/>
     </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
@@ -6797,7 +6803,7 @@
       <c r="Q82" s="2"/>
       <c r="R82" s="2"/>
     </row>
-    <row r="83" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
@@ -6817,7 +6823,7 @@
       <c r="Q83" s="2"/>
       <c r="R83" s="2"/>
     </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -6837,7 +6843,7 @@
       <c r="Q84" s="2"/>
       <c r="R84" s="2"/>
     </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
@@ -6857,7 +6863,7 @@
       <c r="Q85" s="2"/>
       <c r="R85" s="2"/>
     </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -6877,7 +6883,7 @@
       <c r="Q86" s="2"/>
       <c r="R86" s="2"/>
     </row>
-    <row r="87" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -6897,7 +6903,7 @@
       <c r="Q87" s="2"/>
       <c r="R87" s="2"/>
     </row>
-    <row r="88" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -6917,7 +6923,7 @@
       <c r="Q88" s="2"/>
       <c r="R88" s="2"/>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -6937,7 +6943,7 @@
       <c r="Q89" s="2"/>
       <c r="R89" s="2"/>
     </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
@@ -6957,7 +6963,7 @@
       <c r="Q90" s="2"/>
       <c r="R90" s="2"/>
     </row>
-    <row r="91" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -6977,7 +6983,7 @@
       <c r="Q91" s="2"/>
       <c r="R91" s="2"/>
     </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
@@ -6997,7 +7003,7 @@
       <c r="Q92" s="2"/>
       <c r="R92" s="2"/>
     </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -7017,7 +7023,7 @@
       <c r="Q93" s="2"/>
       <c r="R93" s="2"/>
     </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
@@ -7037,7 +7043,7 @@
       <c r="Q94" s="2"/>
       <c r="R94" s="2"/>
     </row>
-    <row r="95" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -7057,7 +7063,7 @@
       <c r="Q95" s="2"/>
       <c r="R95" s="2"/>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -7077,7 +7083,7 @@
       <c r="Q96" s="2"/>
       <c r="R96" s="2"/>
     </row>
-    <row r="97" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -7097,7 +7103,7 @@
       <c r="Q97" s="2"/>
       <c r="R97" s="2"/>
     </row>
-    <row r="98" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -7117,7 +7123,7 @@
       <c r="Q98" s="2"/>
       <c r="R98" s="2"/>
     </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -7137,7 +7143,7 @@
       <c r="Q99" s="2"/>
       <c r="R99" s="2"/>
     </row>
-    <row r="100" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -7167,12 +7173,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E100"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="5" width="20.81640625" style="3" customWidth="1"/>
+    <col min="1" max="5" width="20.77734375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -7189,693 +7195,693 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="9"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
       <c r="E50" s="2"/>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="2"/>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
       <c r="E56" s="2"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2"/>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
       <c r="E58" s="2"/>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
       <c r="E61" s="2"/>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
       <c r="E62" s="2"/>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
       <c r="E63" s="2"/>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
       <c r="E65" s="2"/>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
       <c r="D68" s="2"/>
       <c r="E68" s="2"/>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
       <c r="D69" s="2"/>
       <c r="E69" s="2"/>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
       <c r="D70" s="2"/>
       <c r="E70" s="2"/>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
       <c r="D71" s="2"/>
       <c r="E71" s="2"/>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
       <c r="D72" s="2"/>
       <c r="E72" s="2"/>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
       <c r="D73" s="2"/>
       <c r="E73" s="2"/>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
       <c r="D74" s="2"/>
       <c r="E74" s="2"/>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
       <c r="E75" s="2"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
       <c r="E76" s="2"/>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
       <c r="D77" s="2"/>
       <c r="E77" s="2"/>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
       <c r="E78" s="2"/>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
       <c r="E79" s="2"/>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
       <c r="E80" s="2"/>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
       <c r="D81" s="2"/>
       <c r="E81" s="2"/>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
       <c r="D82" s="2"/>
       <c r="E82" s="2"/>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
       <c r="D83" s="2"/>
       <c r="E83" s="2"/>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
       <c r="D84" s="2"/>
       <c r="E84" s="2"/>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
       <c r="D85" s="2"/>
       <c r="E85" s="2"/>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
       <c r="E86" s="2"/>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
       <c r="E88" s="2"/>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
       <c r="E89" s="2"/>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
       <c r="E90" s="2"/>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
       <c r="D91" s="2"/>
       <c r="E91" s="2"/>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2"/>
       <c r="E92" s="2"/>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
       <c r="D93" s="2"/>
       <c r="E93" s="2"/>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
       <c r="D94" s="2"/>
       <c r="E94" s="2"/>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
       <c r="D95" s="2"/>
       <c r="E95" s="2"/>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
       <c r="D96" s="2"/>
       <c r="E96" s="2"/>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
       <c r="D97" s="2"/>
       <c r="E97" s="2"/>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
       <c r="D98" s="2"/>
       <c r="E98" s="2"/>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
       <c r="D99" s="2"/>
       <c r="E99" s="2"/>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>

</xml_diff>